<commit_message>
raincloud: Add raincloud plot module with QA suite and demo files
</commit_message>
<xml_diff>
--- a/tabtools/demo/table1_sparklines.xlsx
+++ b/tabtools/demo/table1_sparklines.xlsx
@@ -4080,35 +4080,35 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>714375</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
-        <xdr:cNvPicPr>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <twoCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>71437</colOff>
+      <row>3</row>
+      <rowOff>19050</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>785812</colOff>
+      <row>3</row>
+      <rowOff>209550</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Picture 1"/>
+        <cNvPicPr>
           <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
         <a:blip r:embed="rId1"/>
         <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
+      </blipFill>
+      <spPr>
         <a:xfrm>
           <a:off x="685800" y="904875"/>
           <a:ext cx="1219370" cy="1219370"/>
@@ -4116,38 +4116,38 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>714375</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2"/>
-        <xdr:cNvPicPr>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>71437</colOff>
+      <row>4</row>
+      <rowOff>19050</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>785812</colOff>
+      <row>4</row>
+      <rowOff>209550</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Picture 2"/>
+        <cNvPicPr>
           <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
         <a:blip r:embed="rId2"/>
         <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
+      </blipFill>
+      <spPr>
         <a:xfrm>
           <a:off x="685800" y="904875"/>
           <a:ext cx="1219370" cy="1219370"/>
@@ -4155,38 +4155,38 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>714375</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3"/>
-        <xdr:cNvPicPr>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>71437</colOff>
+      <row>5</row>
+      <rowOff>19050</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>785812</colOff>
+      <row>5</row>
+      <rowOff>209550</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Picture 3"/>
+        <cNvPicPr>
           <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
         <a:blip r:embed="rId3"/>
         <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
+      </blipFill>
+      <spPr>
         <a:xfrm>
           <a:off x="685800" y="904875"/>
           <a:ext cx="1219370" cy="1219370"/>
@@ -4194,38 +4194,38 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>714375</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4"/>
-        <xdr:cNvPicPr>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>71437</colOff>
+      <row>6</row>
+      <rowOff>19050</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>785812</colOff>
+      <row>6</row>
+      <rowOff>209550</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Picture 4"/>
+        <cNvPicPr>
           <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
         <a:blip r:embed="rId4"/>
         <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
+      </blipFill>
+      <spPr>
         <a:xfrm>
           <a:off x="685800" y="904875"/>
           <a:ext cx="1219370" cy="1219370"/>
@@ -4233,38 +4233,38 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>714375</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5"/>
-        <xdr:cNvPicPr>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>71437</colOff>
+      <row>7</row>
+      <rowOff>19050</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>785812</colOff>
+      <row>7</row>
+      <rowOff>209550</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Picture 5"/>
+        <cNvPicPr>
           <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
         <a:blip r:embed="rId5"/>
         <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
+      </blipFill>
+      <spPr>
         <a:xfrm>
           <a:off x="685800" y="904875"/>
           <a:ext cx="1219370" cy="1219370"/>
@@ -4272,11 +4272,11 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>